<commit_message>
Add Destinations sheet to packages workbook
Add a second "Destinations" sheet listing the 11 trending destinations:
Destination Name, Price, Destination Image URL, Package Count. Matches
the styling of the Packages sheet (navy header, frozen row, auto-filter).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164FbW6ihQ5PduLzDquHYBA
</commit_message>
<xml_diff>
--- a/flamingo-packages.xlsx
+++ b/flamingo-packages.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Packages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Destinations" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Packages'!$A$1:$H$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Destinations'!$A$1:$D$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +31,11 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
@@ -78,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -100,6 +107,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2247,4 +2257,289 @@
   <autoFilter ref="A1:H42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Destination Name</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Destination Image URL</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Package Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Iceland</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>From $1,741</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/BestSellingDestination/trending-iceland.jpg</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>3+ Packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Scandinavia</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>From $1,341</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/ExploreDestinationByTheme/trending-scandinavia.jpg</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>11+ Packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>From $1,405</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/ExploreDestinationByTheme/trending-spain.jpg</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>12+ Packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>All of Europe</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>From $2,140</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/ExploreDestinationByTheme/trending-all-of-europe.jpg</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>17+ Packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Greece</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>From $1,860</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/ExploreDestinationByTheme/trending-greece.jpg</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>2+ Packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>From $971</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/ExploreDestinationByTheme/trending-south-africa.jpeg</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>18+ Packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>From $1,198</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/ExploreDestinationByTheme/trending-canada.jpg</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>5+ Packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Baku - Azerbaijan</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>From $447</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/ExploreDestinationByTheme/trending-baku.jpg</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>11+ Packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>From $227</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/ExploreDestinationByTheme/trending-Vietnam.jpg</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>31+ Packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>From $347</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/ExploreDestinationByTheme/trending-singapore.jpeg</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>27+ Packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>From $313</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Website/ExploreDestinationByTheme/trending-Malaysia.jpg</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>28+ Packages</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Budget Group column to Packages sheet
Add a "Budget Group" column (Upto 1500 USD / Upto 3500 USD / Upto 5000
USD / Monsoon Special) to the Packages sheet. Packages that appear under
more than one budget group are now listed once per group (45 rows),
sorted by group then name, so each row carries a single clean group value.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164FbW6ihQ5PduLzDquHYBA
</commit_message>
<xml_diff>
--- a/flamingo-packages.xlsx
+++ b/flamingo-packages.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Destinations" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Packages'!$A$1:$H$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Packages'!$A$1:$I$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Destinations'!$A$1:$D$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,19 +21,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -85,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -107,9 +101,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -476,17 +467,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -497,35 +489,40 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Budget Group</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Package Image URL</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>City List</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Flight Included (text)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flight Included?</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Itinerary Length</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
@@ -534,42 +531,47 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Experience Vietnam With Phu Quoc</t>
+          <t>Best Of Baltic Capitals - Sic Tour</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/saigon-municipality-in-vietnam1.jpg</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi (1N), Halong (1N), +3 more</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/keila-joa-castle-1.jpg</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Tallinn (3N), Riga (3N), +1 more</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>$1,255</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
+          <t>$1,378</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
           <t>9N/10D</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Group Tour</t>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Free &amp; Easy – SIC Tour</t>
         </is>
       </c>
     </row>
@@ -581,35 +583,40 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
           <t>https://imgcdn.flamingotravels.co.in/Images/City/hochi-minh-mausoleum.jpg</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Hanoi (2N), Halong (1N), +2 more</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
           <t>$1,135</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>8N/9D</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -623,35 +630,40 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t>https://imgcdn.flamingotravels.co.in/Images/City/one-pillarpagoda-buddhist.jpg</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Ho Chi Minh City (2N), Da Nang (3N), +4 more</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
           <t>$1,305</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>10N/11D</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -660,82 +672,92 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>South East Eminence Singapore Malaysia With Cruise</t>
+          <t>Exotic South Africa - Self Drive</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/wings-of-time-sentosa02.jpg</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Singapore (3N), Cruise (2N), +3 more</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/cap-town-boulders-beach.jpg</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Johannesburg (1N), Knysna (2N), +2 more</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>$1,475</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>8N/9D</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>Group Tour</t>
+          <t>$1,473</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>9N/10D</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Self Drive Tour</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>South East Discovery Singapore Malaysia With Cruise</t>
+          <t>Experience Vietnam With Phu Quoc</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/kl-tower-image-02.jpg</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Singapore (3N), Cruise (2N), +1 more</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/saigon-municipality-in-vietnam1.jpg</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi (1N), Halong (1N), +3 more</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>$1,345</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>8N/9D</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
+          <t>$1,255</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>9N/10D</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -744,166 +766,186 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Glimpse of South Africa - Self Drive</t>
+          <t>Fascinating Spain by Rail</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/ItineraryImage/76_203_cangocaves_1.jpg</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Cape Town (4N), George (3N)</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/sagradafamilia-cover.jpg</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Madrid (2N), Seville (2N), +3 more</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>$966</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>7N/8D</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Self Drive Tour</t>
+          <t>$1,766</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>10N/11D</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Europe By Rail</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Fascinating Spain by Rail</t>
+          <t>Glimpse of South Africa - Self Drive</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/sagradafamilia-cover.jpg</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Madrid (2N), Seville (2N), +3 more</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/ItineraryImage/76_203_cangocaves_1.jpg</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Cape Town (4N), George (3N)</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>$1,766</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>10N/11D</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Europe By Rail</t>
+          <t>$966</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>7N/8D</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Self Drive Tour</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Splendid South Africa - Private Tour</t>
+          <t>Highlights Of Spain By Rail</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/boulders-beach-penguin-colony.jpg</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Johannesburg (1N), Sun City (2N), +2 more</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/visit-royal-palace-of-madrid.jpg</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Madrid (2N), Seville (2N), +2 more</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>$1,705</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>9N/10D</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>Private Van Tour</t>
+          <t>$1,400</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>10N/11D</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Free &amp; Easy – SIC Tour</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Best Of Baltic Capitals - Sic Tour</t>
+          <t>Las Vegas &amp; Surround</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/keila-joa-castle-1.jpg</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Tallinn (3N), Riga (3N), +1 more</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/stratosphere-Tower-Observatory-0.jpg</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Las Vegas (7N)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>$1,378</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>9N/10D</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
+          <t>$1,165</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>7N/8D</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Free &amp; Easy – SIC Tour</t>
         </is>
@@ -912,208 +954,233 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Highlights Of Spain By Rail</t>
+          <t>South East Discovery Singapore Malaysia With Cruise</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/visit-royal-palace-of-madrid.jpg</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Madrid (2N), Seville (2N), +2 more</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/kl-tower-image-02.jpg</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Singapore (3N), Cruise (2N), +1 more</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>$1,400</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>10N/11D</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>Free &amp; Easy – SIC Tour</t>
+          <t>$1,345</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>8N/9D</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Las Vegas &amp; Surround</t>
+          <t>South East Eminence Singapore Malaysia With Cruise</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/stratosphere-Tower-Observatory-0.jpg</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Las Vegas (7N)</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/wings-of-time-sentosa02.jpg</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Singapore (3N), Cruise (2N), +3 more</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>$1,165</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>7N/8D</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Free &amp; Easy – SIC Tour</t>
+          <t>$1,475</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>8N/9D</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Exotic South Africa - Self Drive</t>
+          <t>Splendid South Africa - Private Tour</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/cap-town-boulders-beach.jpg</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Johannesburg (1N), Knysna (2N), +2 more</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 1500 USD</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/boulders-beach-penguin-colony.jpg</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Johannesburg (1N), Sun City (2N), +2 more</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>$1,473</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
+          <t>$1,705</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
           <t>9N/10D</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>Self Drive Tour</t>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Private Van Tour</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>European Elements</t>
+          <t>Amazing Australia With Heavenly Hamilton</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/Madame-Tussauds.jpg</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>London (2N), Paris (2N), +6 more</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 3500 USD</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/48543073737_b0f1e92795_o.jpg</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Gold Coast (4N), Hamilton Island (3N), +3 more</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>$3,815</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
+          <t>$2,610</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>14N/15D</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Group Tour</t>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Free &amp; Easy – SIC Tour</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Experience Canadian Rockies</t>
+          <t>Dreams 1 Singapore Malaysia with 2 Nights Cruise</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/moraine-lake-banffnationalpark.jpg</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Calgary (1N), Canmore (2N), +4 more</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 3500 USD</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/Singapore-city-skyline.JPG</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur (1N), Genting Highlands (1N), +3 more</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>$3,765</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
+          <t>$1,565</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
           <t>9N/10D</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1122,40 +1189,45 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Experience New Zealand with Australia</t>
+          <t>European Dreams</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/melbourne-aerial-view-001.jpg</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Auckland (1N), Rotorua (2N), +7 more</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Internal Flight Included</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Upto 3500 USD</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/vevey-citycentreview.jpg</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Paris (3N), Lausanne (1N), +1 more</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>$5,575</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>18N/19D</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
+          <t>$2,135</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>7N/8D</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1164,40 +1236,45 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>South African Lite Tour</t>
+          <t>Exotic Africa With Victoria Falls with Chef</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/table-mountain-from-harbour.jpg</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Cape Town (4N), George (3N), +1 more</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
+          <t>Upto 3500 USD</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/ItineraryImage/victoria- Fall.jpg</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Cape Town (4N), George (3N), +4 more</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Internal Flight Included</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>$2,095</t>
-        </is>
-      </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>8N/9D</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
+          <t>$3,715</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>13N/14D</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1206,40 +1283,45 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Discover South Korea</t>
+          <t>Experience Canadian Rockies</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/bukchon-hanok-village-1.jpg</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Seoul (2N), Busan (2N), +1 more</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 3500 USD</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/moraine-lake-banffnationalpark.jpg</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Calgary (1N), Canmore (2N), +4 more</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>$1,745</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>6N/7D</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
+          <t>$3,765</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>9N/10D</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1248,124 +1330,139 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>American Explorer</t>
+          <t>Naturally New Zealand With Beautiful Bora Bora Self Drive</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/usa-package-jip.jpg</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>New York City (2N), Washington (1N), +4 more</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Internal Flight Included</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Upto 3500 USD</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Fallback/flamingo_fallback_250x120.jpg</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Auckland (1N), Rotorua (3N), +6 more</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>$4,445</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>12N/13D</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>Group Tour</t>
+          <t>$2,947</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>14N/15D</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Self Drive Tour</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Discovery Bali With Mara River Safari</t>
+          <t>Stunning South Africa – Private Tour</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/tanah-lot-temple02.JPG</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Bali Island (2N), Bali Island (2N), +2 more</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 3500 USD</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/Fallback/flamingo_fallback_250x120.jpg</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Johannesburg (1N), Kruger National Park (2N), +4 more</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>$775</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>6N/7D</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Group Tour</t>
+          <t>$2,197</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>11N/12D</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Private Van Tour</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Escape Singapore Malaysia with Langkawi</t>
+          <t>Vietnam &amp; Cambodia Highlights</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/batu-caves--00.jpg</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Kuala Lumpur (1N), Langkawi (3N), +2 more</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 3500 USD</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/hanoi.jpg</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi (2N), Halong (1N), +3 more</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>$1,445</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>9N/10D</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
+          <t>$1,935</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>12N/13D</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1374,40 +1471,45 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Discovery Vietnam With Ninh Binh - Senior Citizen Special Tour</t>
+          <t>Whole of South Africa 3 with Chef</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/halongbay-daytrip.jpg</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City (2N), Da Nang (3N), +2 more</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 3500 USD</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/Game Drive Experience.jpg</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Cape Town (4N), George (3N), +4 more</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Internal Flight Included</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>$1,025</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>8N/9D</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
+          <t>$3,495</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>13N/14D</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1416,124 +1518,139 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Dazzling Singapore</t>
+          <t>American Escape</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/universal-studio-singapre.jpg</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Singapore (3N), Singapore (1N)</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/statue-of-liberty.jpg</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>San Francisco (2N), Los Angeles (2N), +4 more</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Internal Flight Included</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>$931</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>4N/5D</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>Private Van Tour</t>
+          <t>$4,145</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>12N/13D</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Naturally New Zealand - Self Drive</t>
+          <t>American Experience East &amp; West</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/agrodome-sheep-show-001.jpg</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Auckland (1N), Rotorua (2N), +4 more</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/new-jersey-1.jpg</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>New York City (2N), Washington (1N), +4 more</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Internal Flight Included</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>$1,348</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>9N/10D</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Self Drive Tour</t>
+          <t>$4,645</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>12N/13D</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Vietnam &amp; Cambodia Highlights</t>
+          <t>American Explorer</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/hanoi.jpg</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Hanoi (2N), Halong (1N), +3 more</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/usa-package-jip.jpg</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>New York City (2N), Washington (1N), +4 more</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Internal Flight Included</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>$1,935</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
+          <t>$4,445</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
           <t>12N/13D</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1542,40 +1659,45 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Whole of South Africa 3 with Chef</t>
+          <t>Captivating Canadian Rockies</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/Game Drive Experience.jpg</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Cape Town (4N), George (3N), +4 more</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Internal Flight Included</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/sulphur-mountain-anff.png</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Calgary (1N), Banff (2N), +4 more</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>$3,495</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>13N/14D</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
+          <t>$3,875</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>9N/10D</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1584,40 +1706,45 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Dreams 1 Singapore Malaysia with 2 Nights Cruise</t>
+          <t>European Elegance (Hook on to Exotic)</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/Singapore-city-skyline.JPG</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Kuala Lumpur (1N), Genting Highlands (1N), +3 more</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/arc-de-triomphe-aerial-view.jpg</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Paris (3N), Lausanne (2N), +5 more</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>$1,565</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>9N/10D</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
+          <t>$3,675</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>12N/13D</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1626,40 +1753,45 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Exotic Africa With Victoria Falls with Chef</t>
+          <t>European Elements</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/ItineraryImage/victoria- Fall.jpg</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Cape Town (4N), George (3N), +4 more</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Internal Flight Included</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/Madame-Tussauds.jpg</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>London (2N), Paris (2N), +6 more</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>$3,715</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>13N/14D</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
+          <t>$3,815</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>14N/15D</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1668,40 +1800,45 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>European Dreams</t>
+          <t>European Euphoria</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/vevey-citycentreview.jpg</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Paris (3N), Lausanne (1N), +1 more</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/visit-nestle-cailler-chocolate-factorq.jpg</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Paris (3N), Amsterdam (2N), +6 more</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>$2,135</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>7N/8D</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
+          <t>$3,645</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>13N/14D</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1710,250 +1847,280 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Amazing Australia With Heavenly Hamilton</t>
+          <t>Experience Australia Tour Perth Special</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/48543073737_b0f1e92795_o.jpg</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Gold Coast (4N), Hamilton Island (3N), +3 more</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/great ocean road-002.jpg</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Perth (3N), Cairns (2N), +2 more</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Internal Flight Included</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>$2,610</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>14N/15D</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>Free &amp; Easy – SIC Tour</t>
+          <t>$3,755</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>11N/12D</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Naturally New Zealand With Beautiful Bora Bora Self Drive</t>
+          <t>Experience New Zealand with Australia</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/Fallback/flamingo_fallback_250x120.jpg</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Auckland (1N), Rotorua (3N), +6 more</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/melbourne-aerial-view-001.jpg</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Auckland (1N), Rotorua (2N), +7 more</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>Internal Flight Included</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>$2,947</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>14N/15D</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>Self Drive Tour</t>
+          <t>$5,575</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>18N/19D</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Stunning South Africa – Private Tour</t>
+          <t>Interesting Iceland - Chef Assisted Tour</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/Fallback/flamingo_fallback_250x120.jpg</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Johannesburg (1N), Kruger National Park (2N), +4 more</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/seljalandsfoss-waterfalls-1.jpg</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Reykjavik (2N), Akyureri (2N), +3 more</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>$2,197</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>11N/12D</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>Private Van Tour</t>
+          <t>$4,115</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>9N/10D</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Captivating Canadian Rockies</t>
+          <t>Kenya With Tanzania Migration Special</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/sulphur-mountain-anff.png</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Calgary (1N), Banff (2N), +4 more</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/kenya-1.jpg</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Nairobi (1N), Masai Mara (2N), +5 more</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>$3,875</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>9N/10D</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>Group Tour</t>
+          <t>$4,589</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>10N/11D</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>Fixed Departure</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>UK Scotland And Ireland Tour</t>
+          <t>Naturally New Zealand With Pure Pods  Private</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/national-museum-of-dublin-001.jpg</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>London (3N), Cardiff (1N), +5 more</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/cathedral-cove-001.jpg</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Auckland (1N), Paihia (2N), +10 more</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>$3,955</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>13N/14D</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>Group Tour</t>
+          <t>$4,565</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>22N/23D</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Private Van Tour</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Interesting Iceland - Chef Assisted Tour</t>
+          <t>UK Scotland And Ireland Tour</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/seljalandsfoss-waterfalls-1.jpg</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Reykjavik (2N), Akyureri (2N), +3 more</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Upto 5000 USD</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/national-museum-of-dublin-001.jpg</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>London (3N), Cardiff (1N), +5 more</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>$4,115</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>9N/10D</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
+          <t>$3,955</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>13N/14D</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -1962,40 +2129,45 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>American Escape</t>
+          <t>American Explorer</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/statue-of-liberty.jpg</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>San Francisco (2N), Los Angeles (2N), +4 more</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/usa-package-jip.jpg</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>New York City (2N), Washington (1N), +4 more</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>Internal Flight Included</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>$4,145</t>
-        </is>
-      </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
+          <t>$4,445</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
           <t>12N/13D</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
+      <c r="I36" s="3" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -2004,82 +2176,92 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>American Experience East &amp; West</t>
+          <t>Dazzling Singapore</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/new-jersey-1.jpg</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>New York City (2N), Washington (1N), +4 more</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>Internal Flight Included</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/universal-studio-singapre.jpg</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Singapore (3N), Singapore (1N)</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>$4,645</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>12N/13D</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>Group Tour</t>
+          <t>$931</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>4N/5D</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Private Van Tour</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>European Euphoria</t>
+          <t>Discover South Korea</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/visit-nestle-cailler-chocolate-factorq.jpg</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Paris (3N), Amsterdam (2N), +6 more</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/bukchon-hanok-village-1.jpg</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Seoul (2N), Busan (2N), +1 more</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>$3,645</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>13N/14D</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
+          <t>$1,745</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>6N/7D</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -2088,40 +2270,45 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>European Elegance (Hook on to Exotic)</t>
+          <t>Discovery Bali With Mara River Safari</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/arc-de-triomphe-aerial-view.jpg</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Paris (3N), Lausanne (2N), +5 more</t>
-        </is>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/tanah-lot-temple02.JPG</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Bali Island (2N), Bali Island (2N), +2 more</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>$3,675</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>12N/13D</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
+          <t>$775</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>6N/7D</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -2130,40 +2317,45 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Experience Australia Tour Perth Special</t>
+          <t>Discovery Vietnam With Ninh Binh - Senior Citizen Special Tour</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/great ocean road-002.jpg</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Perth (3N), Cairns (2N), +2 more</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>Internal Flight Included</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/halongbay-daytrip.jpg</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City (2N), Da Nang (3N), +2 more</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>$3,755</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>11N/12D</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
+          <t>$1,025</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>8N/9D</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
         <is>
           <t>Group Tour</t>
         </is>
@@ -2172,89 +2364,287 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Naturally New Zealand With Pure Pods  Private</t>
+          <t>Escape Singapore Malaysia with Langkawi</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/cathedral-cove-001.jpg</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>Auckland (1N), Paihia (2N), +10 more</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/batu-caves--00.jpg</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur (1N), Langkawi (3N), +2 more</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>$4,565</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>22N/23D</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>Private Van Tour</t>
+          <t>$1,445</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>9N/10D</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Kenya With Tanzania Migration Special</t>
+          <t>European Elements</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>https://imgcdn.flamingotravels.co.in/Images/City/kenya-1.jpg</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Nairobi (1N), Masai Mara (2N), +5 more</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>Flight Not Included</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/Madame-Tussauds.jpg</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>London (2N), Paris (2N), +6 more</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>$4,589</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>10N/11D</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>Fixed Departure</t>
+          <t>$3,815</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>14N/15D</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Experience Canadian Rockies</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/moraine-lake-banffnationalpark.jpg</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Calgary (1N), Canmore (2N), +4 more</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>$3,765</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>9N/10D</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Experience New Zealand with Australia</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/melbourne-aerial-view-001.jpg</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Auckland (1N), Rotorua (2N), +7 more</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Internal Flight Included</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>$5,575</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>18N/19D</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Naturally New Zealand - Self Drive</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/agrodome-sheep-show-001.jpg</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Auckland (1N), Rotorua (2N), +4 more</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>Flight Not Included</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>$1,348</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>9N/10D</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Self Drive Tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>South African Lite Tour</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Monsoon Special</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>https://imgcdn.flamingotravels.co.in/Images/City/table-mountain-from-harbour.jpg</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Cape Town (4N), George (3N), +1 more</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Internal Flight Included</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>$2,095</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>8N/9D</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Group Tour</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H42"/>
+  <autoFilter ref="A1:I46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2275,22 +2665,22 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Destination Name</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Destination Image URL</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Package Count</t>
         </is>

</xml_diff>

<commit_message>
Use full city lists from embedded package data
Replace the truncated card city lists ("Hanoi, Halong, +3 more") with
the complete lists parsed from the __NEXT_DATA__ JSON in the source HTML
files (e.g. "Hanoi (2N), Halong (1N), Da Nang (3N), Ho Chi Minh City (2N)").
All 45 package rows matched by name; city lists are consistent across
budget groups.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164FbW6ihQ5PduLzDquHYBA
</commit_message>
<xml_diff>
--- a/flamingo-packages.xlsx
+++ b/flamingo-packages.xlsx
@@ -472,8 +472,8 @@
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -546,7 +546,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Tallinn (3N), Riga (3N), +1 more</t>
+          <t>Tallinn (3N), Riga (3N), Vilnius (3N)</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Hanoi (2N), Halong (1N), +2 more</t>
+          <t>Hanoi (2N), Halong (1N), Da Nang (3N), Ho Chi Minh City (2N)</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City (2N), Da Nang (3N), +4 more</t>
+          <t>Ho Chi Minh City (2N), Da Nang (3N), Hanoi (1N), Sa Pa (2N), Hanoi (1N), Halong (1N)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Johannesburg (1N), Knysna (2N), +2 more</t>
+          <t>Johannesburg (1N), Knysna (2N), Private Game Reserve (2N), Cape Town (4N)</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Hanoi (1N), Halong (1N), +3 more</t>
+          <t>Hanoi (1N), Halong (1N), Da Nang (3N), Phu Quoc (3N), Ho Chi Minh City (1N)</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Madrid (2N), Seville (2N), +3 more</t>
+          <t>Madrid (2N), Seville (2N), Valencia (1N), Ibiza (2N), Barcelona (3N)</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Madrid (2N), Seville (2N), +2 more</t>
+          <t>Madrid (2N), Seville (2N), Malaga (3N), Barcelona (3N)</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Singapore (3N), Cruise (2N), +1 more</t>
+          <t>Singapore (3N), Cruise (2N), Kuala Lumpur (3N)</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Singapore (3N), Cruise (2N), +3 more</t>
+          <t>Singapore (2N), Cruise (2N), Singapore (1N), Kuala Lumpur (1N), Genting Highlands (1N), Kuala Lumpur (1N)</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Johannesburg (1N), Sun City (2N), +2 more</t>
+          <t>Johannesburg (1N), Sun City (2N), George (3N), Cape Town (3N)</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Gold Coast (4N), Hamilton Island (3N), +3 more</t>
+          <t>Gold Coast (4N), Hamilton Island (3N), Sydney (4N), Melbourne (2N), Melbourne (1N)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Kuala Lumpur (1N), Genting Highlands (1N), +3 more</t>
+          <t>Kuala Lumpur (1N), Genting Highlands (1N), Sunway Lagoon (2N), Cruise (2N), Singapore (3N)</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Paris (3N), Lausanne (1N), +1 more</t>
+          <t>Paris (3N), Lausanne (1N), Zurich (3N)</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Cape Town (4N), George (3N), +4 more</t>
+          <t>Cape Town (4N), George (3N), Johannesburg (1N), Kruger National Park (2N), Johannesburg (1N), Victoria Falls ZI (2N)</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Calgary (1N), Canmore (2N), +4 more</t>
+          <t>Calgary (1N), Canmore (2N), Hinton (2N), Kamloops (1N), Victoria CN (1N), Vancouver (2N)</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Auckland (1N), Rotorua (3N), +6 more</t>
+          <t>Auckland (1N), Rotorua (3N), Auckland (1N), Queenstown (3N), Twizel (1N), Christchurch (1N), Tahiti (1N), Bora Bora (3N)</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Johannesburg (1N), Kruger National Park (2N), +4 more</t>
+          <t>Johannesburg (1N), Kruger National Park (2N), Johannesburg (1N), Knysna (2N), Hermanus (2N), Cape Town (3N)</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Hanoi (2N), Halong (1N), +3 more</t>
+          <t>Hanoi (2N), Halong (1N), Da Nang (3N), Ho Chi Minh City (3N), Siem Reap (3N)</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Cape Town (4N), George (3N), +4 more</t>
+          <t>Cape Town (4N), George (3N), Johannesburg (1N), Kruger National Park (2N), Johannesburg (1N), Sun City (2N)</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>San Francisco (2N), Los Angeles (2N), +4 more</t>
+          <t>San Francisco (2N), Los Angeles (2N), Las Vegas (3N), Niagara Falls USA (2N), Washington (1N), New Jersey (2N)</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>New York City (2N), Washington (1N), +4 more</t>
+          <t>New York City (2N), Washington (1N), Niagara Falls USA (2N), Las Vegas (3N), Los Angeles (2N), San Francisco (2N)</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>New York City (2N), Washington (1N), +4 more</t>
+          <t>New York City (2N), Washington (1N), Niagara Falls USA (2N), Las Vegas (3N), Los Angeles (2N), San Francisco (2N)</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Calgary (1N), Banff (2N), +4 more</t>
+          <t>Calgary (1N), Banff (2N), Jasper (2N), Kamloops (1N), Whistler (1N), Vancouver (2N)</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Paris (3N), Lausanne (2N), +5 more</t>
+          <t>Paris (3N), Lausanne (2N), Engelberg (2N), Zurich (1N), Innsbruck (1N), Salzburg (1N), Vienna (2N)</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>London (2N), Paris (2N), +6 more</t>
+          <t>London (2N), Paris (2N), Amsterdam (2N), Heppenheim (1N), Zurich (3N), Innsbruck (1N), Padova (1N), Arezzo (2N)</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Paris (3N), Amsterdam (2N), +6 more</t>
+          <t>Paris (3N), Amsterdam (2N), Mannheim (1N), Munich (1N), Innsbruck (1N), Engelberg (2N), Lausanne (2N), Zurich (1N)</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Perth (3N), Cairns (2N), +2 more</t>
+          <t>Perth (3N), Cairns (2N), Melbourne (3N), Sydney (3N)</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Auckland (1N), Rotorua (2N), +7 more</t>
+          <t>Auckland (1N), Rotorua (2N), Auckland (1N), Queenstown (4N), Twizel (1N), Christchurch (1N), Sydney (3N), Cairns (2N), Melbourne (3N)</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Reykjavik (2N), Akyureri (2N), +3 more</t>
+          <t>Reykjavik (2N), Akyureri (2N), Borgarnes (2N), Vik I Myrdal (2N), Keflavik (1N)</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Nairobi (1N), Masai Mara (2N), +5 more</t>
+          <t>Nairobi (1N), Masai Mara (2N), Naivasha (1N), Amboseli National Park (2N), Lake Manyara National Park (1N), Serengeti (2N), Lake Manyara National Park (1N)</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Auckland (1N), Paihia (2N), +10 more</t>
+          <t>Auckland (1N), Paihia (2N), Auckland (1N), Whitianga (2N), Rotorua (4N), Auckland (1N), Kaikoura (1N), Pure Pods (1N), Franz Josef (2N), Queenstown (4N), Lake Tekapo (1N), Christchurch (2N)</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>London (3N), Cardiff (1N), +5 more</t>
+          <t>London (3N), Cardiff (1N), Manchester (1N), Blackpool (1N), Glasgow (3N), Belfast (2N), Dublin (2N)</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>New York City (2N), Washington (1N), +4 more</t>
+          <t>New York City (2N), Washington (1N), Niagara Falls USA (2N), Las Vegas (3N), Los Angeles (2N), San Francisco (2N)</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Seoul (2N), Busan (2N), +1 more</t>
+          <t>Seoul (2N), Busan (2N), Seoul (2N)</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Bali Island (2N), Bali Island (2N), +2 more</t>
+          <t>Bali Island (2N), Bali Island (2N), Bali Island (1N), Bali Island (1N)</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City (2N), Da Nang (3N), +2 more</t>
+          <t>Ho Chi Minh City (2N), Da Nang (3N), Hanoi (2N), Halong (1N)</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Kuala Lumpur (1N), Langkawi (3N), +2 more</t>
+          <t>Kuala Lumpur (1N), Langkawi (3N), Kuala Lumpur (2N), Singapore (3N)</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>London (2N), Paris (2N), +6 more</t>
+          <t>London (2N), Paris (2N), Amsterdam (2N), Heppenheim (1N), Zurich (3N), Innsbruck (1N), Padova (1N), Arezzo (2N)</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Calgary (1N), Canmore (2N), +4 more</t>
+          <t>Calgary (1N), Canmore (2N), Hinton (2N), Kamloops (1N), Victoria CN (1N), Vancouver (2N)</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
@@ -2520,7 +2520,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Auckland (1N), Rotorua (2N), +7 more</t>
+          <t>Auckland (1N), Rotorua (2N), Auckland (1N), Queenstown (4N), Twizel (1N), Christchurch (1N), Sydney (3N), Cairns (2N), Melbourne (3N)</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Auckland (1N), Rotorua (2N), +4 more</t>
+          <t>Auckland (1N), Rotorua (2N), Auckland (1N), Queenstown (3N), Twizel (1N), Christchurch (1N)</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Cape Town (4N), George (3N), +1 more</t>
+          <t>Cape Town (4N), George (3N), Johannesburg (1N)</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Merge consecutive duplicate cities in City List
Collapse consecutive same-city entries by summing their nights (e.g.
"Singapore (3N), Singapore (1N)" -> "Singapore (4N)"). Non-consecutive
repeats are left unchanged. Affects 3 package rows: Discovery Bali With
Mara River Safari, Dazzling Singapore, and Amazing Australia With
Heavenly Hamilton.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164FbW6ihQ5PduLzDquHYBA
</commit_message>
<xml_diff>
--- a/flamingo-packages.xlsx
+++ b/flamingo-packages.xlsx
@@ -1110,7 +1110,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Gold Coast (4N), Hamilton Island (3N), Sydney (4N), Melbourne (2N), Melbourne (1N)</t>
+          <t>Gold Coast (4N), Hamilton Island (3N), Sydney (4N), Melbourne (3N)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Singapore (3N), Singapore (1N)</t>
+          <t>Singapore (4N)</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Bali Island (2N), Bali Island (2N), Bali Island (1N), Bali Island (1N)</t>
+          <t>Bali Island (6N)</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">

</xml_diff>